<commit_message>
client_level_export_server.R - Stop deleting 'Instructions' sheet for the system exits download
CLE Instructions and Data Dictionary.xlsx
- modifications made to Instructions sheet
</commit_message>
<xml_diff>
--- a/www/CLE Instructions and Data Dictionary.xlsx
+++ b/www/CLE Instructions and Data Dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\projects\CE_Data_Toolkit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBE5F895-089F-452D-80B3-74732EC7DA0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90FC8678-A985-46AF-BCC0-C9C9F4153BE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3912" yWindow="1680" windowWidth="17280" windowHeight="9024" firstSheet="1" activeTab="1" xr2:uid="{51E25282-ACA6-44F1-BA60-C197611A1412}"/>
+    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="9024" firstSheet="1" activeTab="1" xr2:uid="{51E25282-ACA6-44F1-BA60-C197611A1412}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="4" r:id="rId1"/>
@@ -594,9 +594,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">4) Monthly Statuses </t>
-  </si>
-  <si>
     <t>The Monthly Statuses tab shows who was housed during the report period, who had at least one system exit to permanent housing during the report period, and the end-of-the-month system status for every client included in the Client Details tab. This allows users to see client outcomes, highlighting changes in system status over the report period. There is one row per client. A blank monthly status indicates the client was not active during that month.</t>
   </si>
   <si>
@@ -643,9 +640,6 @@
       </rPr>
       <t>identifies clients who either moved into housing or exited the system to a permanent destination by the end of the report period</t>
     </r>
-  </si>
-  <si>
-    <t>5) Adjusted Enrollments</t>
   </si>
   <si>
     <t>This tab lists enrollments that had date adjusments for the purposes of Eva's system performance logic. For example, non-residential enrollments without an Exit Date during the report period had their Exit Date reset with a buffer after theEntry Date or last Current Living Situation record (whichever was later).</t>
@@ -867,6 +861,12 @@
   </si>
   <si>
     <t>LH_Dates is an Eva-defined variable. This field lists dates during the enrollment where the client was experincing literal homelessness. Dates may include an Entry Date with a literally homeless Prior Living Situation, Bed-Night Dates for night-by-night enrollments, and Current Living Situation records with a literally homeless living situation.</t>
+  </si>
+  <si>
+    <t>4) Monthly Statuses (System Overview Only)</t>
+  </si>
+  <si>
+    <t>5) Adjusted Enrollments (System Overview Only)</t>
   </si>
 </sst>
 </file>
@@ -1483,19 +1483,12 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
-        <color rgb="FF9C5700"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1511,11 +1504,18 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2047,13 +2047,13 @@
     </row>
     <row r="34" spans="1:2" ht="18" x14ac:dyDescent="0.3">
       <c r="A34" s="10" t="s">
-        <v>117</v>
+        <v>163</v>
       </c>
       <c r="B34" s="8"/>
     </row>
     <row r="35" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B35" s="8"/>
     </row>
@@ -2069,19 +2069,19 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B38" s="8"/>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B39" s="8"/>
     </row>
     <row r="40" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B40" s="8"/>
     </row>
@@ -2091,13 +2091,13 @@
     </row>
     <row r="42" spans="1:2" ht="18" x14ac:dyDescent="0.3">
       <c r="A42" s="10" t="s">
-        <v>122</v>
+        <v>164</v>
       </c>
       <c r="B42" s="8"/>
     </row>
     <row r="43" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B43" s="8"/>
     </row>
@@ -2113,13 +2113,13 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" s="11" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B46" s="8"/>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B47" s="8"/>
     </row>
@@ -2224,13 +2224,13 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -2290,13 +2290,13 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B14" t="s">
         <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -2312,13 +2312,13 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B16" t="s">
         <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -2334,24 +2334,24 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B18" t="s">
         <v>12</v>
       </c>
       <c r="C18" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B19" t="s">
         <v>12</v>
       </c>
       <c r="C19" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -2367,13 +2367,13 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B21" t="s">
         <v>12</v>
       </c>
       <c r="C21" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -2389,13 +2389,13 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B23" t="s">
         <v>12</v>
       </c>
       <c r="C23" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -2411,35 +2411,35 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B25" t="s">
         <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B26" t="s">
         <v>12</v>
       </c>
       <c r="C26" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B27" t="s">
         <v>12</v>
       </c>
       <c r="C27" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -2499,13 +2499,13 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B33" t="s">
         <v>12</v>
       </c>
       <c r="C33" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -2543,35 +2543,35 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B37" t="s">
         <v>12</v>
       </c>
       <c r="C37" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B38" t="s">
         <v>12</v>
       </c>
       <c r="C38" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B39" t="s">
         <v>12</v>
       </c>
       <c r="C39" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -2670,7 +2670,7 @@
         <v>64</v>
       </c>
       <c r="C48" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
@@ -2703,7 +2703,7 @@
         <v>64</v>
       </c>
       <c r="C51" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
@@ -2714,7 +2714,7 @@
         <v>64</v>
       </c>
       <c r="C52" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
@@ -2769,7 +2769,7 @@
         <v>80</v>
       </c>
       <c r="C57" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
@@ -2802,7 +2802,7 @@
         <v>80</v>
       </c>
       <c r="C60" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
@@ -2813,29 +2813,29 @@
         <v>80</v>
       </c>
       <c r="C61" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
+        <v>158</v>
+      </c>
+      <c r="B62" t="s">
+        <v>159</v>
+      </c>
+      <c r="C62" t="s">
         <v>160</v>
-      </c>
-      <c r="B62" t="s">
-        <v>161</v>
-      </c>
-      <c r="C62" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B63" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C63" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -7671,16 +7671,16 @@
     <row r="1" s="13" customFormat="1" ht="15.6" x14ac:dyDescent="0.3"/>
   </sheetData>
   <conditionalFormatting sqref="E1:P1048576">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Inactive">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Inactive">
       <formula>NOT(ISERROR(SEARCH("Inactive",E1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Exited">
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Exited">
       <formula>NOT(ISERROR(SEARCH("Exited",E1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Homeless">
+    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="Homeless">
       <formula>NOT(ISERROR(SEARCH("Homeless",E1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Housed">
+    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="Housed">
       <formula>NOT(ISERROR(SEARCH("Housed",E1)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>